<commit_message>
Corrige entradas para 17 e fecha balanco exato (323); adiciona secao de metodologia
</commit_message>
<xml_diff>
--- a/Conciliacao_DRE_Agosto_x_Folha_Setembro.xlsx
+++ b/Conciliacao_DRE_Agosto_x_Folha_Setembro.xlsx
@@ -450,12 +450,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="47" customWidth="1" min="3" max="3"/>
+    <col width="53" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
@@ -571,24 +571,58 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>PAMELA IRIS GREGORIO IBARRA aparece 2x</t>
+          <t>1 linha(s) excedente(s) por duplicidade</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Reconciliacao</t>
+          <t>Reconciliacao (subtotal)</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>328 - 23 + 16 = 321</t>
+          <t>328 - 23 + 17 = 322</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Aproxima de 322/323 (duplicata na folha)</t>
+          <t>DRE menos saidas mais entradas</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Reconciliacao (final)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>322 + 1 = 323</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Igual ao total real da folha (323) - balanco fecha</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Metodo de cruzamento</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Nome completo normalizado</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Sem acentos, maiusculas, espacos normalizados</t>
         </is>
       </c>
     </row>
@@ -941,7 +975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1050,11 +1084,11 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>FERNANDO ESTEVES ARRUDA</t>
+          <t>FERNANDA DE MORAES SILVA</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>79</v>
+        <v>299</v>
       </c>
     </row>
     <row r="9">
@@ -1063,11 +1097,11 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>ISABELLA STODIEK</t>
+          <t>FERNANDO ESTEVES ARRUDA</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>324</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10">
@@ -1076,11 +1110,11 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>LARISSA STEPHANI OLIVEIRA FREITAS</t>
+          <t>ISABELLA STODIEK</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>294</v>
+        <v>324</v>
       </c>
     </row>
     <row r="11">
@@ -1089,11 +1123,11 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>LUCAS MATHEUS DA SILVA PEÇANHA</t>
+          <t>LARISSA STEPHANI OLIVEIRA FREITAS</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>158</v>
+        <v>294</v>
       </c>
     </row>
     <row r="12">
@@ -1102,11 +1136,11 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>MARIA EDUARDA COELHO BARBOSA ROCHA</t>
+          <t>LUCAS MATHEUS DA SILVA PEÇANHA</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>178</v>
+        <v>158</v>
       </c>
     </row>
     <row r="13">
@@ -1115,11 +1149,11 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>PEDRO HYPOLITO NOGUEIRA</t>
+          <t>MARIA EDUARDA COELHO BARBOSA ROCHA</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>209</v>
+        <v>178</v>
       </c>
     </row>
     <row r="14">
@@ -1128,11 +1162,11 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>RAFAEL ALVES PINHEIRO</t>
+          <t>PEDRO HYPOLITO NOGUEIRA</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>213</v>
+        <v>209</v>
       </c>
     </row>
     <row r="15">
@@ -1141,11 +1175,11 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>RAPHAEL CARDIM CALVET</t>
+          <t>RAFAEL ALVES PINHEIRO</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>219</v>
+        <v>213</v>
       </c>
     </row>
     <row r="16">
@@ -1154,11 +1188,11 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>RENAN MARTINS DOS SANTOS</t>
+          <t>RAPHAEL CARDIM CALVET</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>223</v>
+        <v>219</v>
       </c>
     </row>
     <row r="17">
@@ -1167,10 +1201,23 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
+          <t>RENAN MARTINS DOS SANTOS</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
           <t>ROBERTA RIBEIRO VICENTE CAMPIONI</t>
         </is>
       </c>
-      <c r="C17" s="3" t="n">
+      <c r="C18" s="3" t="n">
         <v>319</v>
       </c>
     </row>

</xml_diff>